<commit_message>
Actualización extracción de tablas SIPLAN
</commit_message>
<xml_diff>
--- a/notebooks/datos/operaciones_siplan.xlsx
+++ b/notebooks/datos/operaciones_siplan.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL47"/>
+  <dimension ref="A1:AL70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7693,6 +7693,3434 @@
         </is>
       </c>
       <c r="AL47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>6 GESTIÓN HUMANA</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2 Integridad</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>75.00%</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Apoyar actividades para implementar caja de herramientas del código de integridad según cronograma</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Caja de herramientas del Código de integridad implementado</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q48" t="n">
+        <v>0</v>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y48" t="inlineStr"/>
+      <c r="Z48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC48" t="inlineStr"/>
+      <c r="AD48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE48" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG48" t="inlineStr">
+        <is>
+          <t>Mediante memorando 20251-V-BOG-030813 de fecha 15 mayo 2025 y 20251-V-BOG-043356 de fehca 20 junio de 2025</t>
+        </is>
+      </c>
+      <c r="AH48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI48" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK48" t="inlineStr">
+        <is>
+          <t>No se encuentra ninguna observación</t>
+        </is>
+      </c>
+      <c r="AL48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>6 GESTIÓN HUMANA</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2 Integridad</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>75.00%</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Apoyar actividades para implementar acciones orientadas al fortalecimiento de la política de transversalización de Equidad de Género y articulación con el Sello Equipares Público</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Actividades orientadas al fortalecimiento de la política de transversalización de Equidad de Género implementadas y con informe de seguimiento</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M49" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O49" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q49" t="n">
+        <v>0</v>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="X49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y49" t="inlineStr"/>
+      <c r="Z49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC49" t="inlineStr"/>
+      <c r="AD49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE49" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG49" t="inlineStr">
+        <is>
+          <t>Mediante memorando 20251-V-BOG-030813 de fecha 15 mayo 2025 y 20251-V-BOG-043356 de fehca 20 junio de 2025</t>
+        </is>
+      </c>
+      <c r="AH49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI49" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK49" t="inlineStr">
+        <is>
+          <t>No se encuentra ninguna observación</t>
+        </is>
+      </c>
+      <c r="AL49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>15 CONTROL DISCIPLINARIO</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>80 Talento Humano</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>75.00%</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Apoyar actividades para implementar un plan de trabajo orientado a la identificación del perfil cultural de la organización.</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Plan de trabajo de cultura organizacional implementado y con informes de seguimiento trimestral</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M50" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O50" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q50" t="n">
+        <v>0</v>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X50" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y50" t="inlineStr"/>
+      <c r="Z50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC50" t="inlineStr"/>
+      <c r="AD50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE50" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG50" t="inlineStr">
+        <is>
+          <t>El día 4 de julio de 2025 se realizó actividad de comunicación efectiva y escucha activa, muro de gratitud y el 25 de septiembre de 2025, se hace actividades de integración con toda la subdirección</t>
+        </is>
+      </c>
+      <c r="AH50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI50" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK50" t="inlineStr">
+        <is>
+          <t>No se encuentra ninguna observación</t>
+        </is>
+      </c>
+      <c r="AL50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>13 DIRECCIONAMIENTO ESTRATÉGICO Y PLANEACIÓN INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>1 Planeación Institucional</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Formular oportunamente los plan operativo del grupo</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>plan operativo formulado</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="M51" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="O51" t="n">
+        <v>0</v>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Q51" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="X51" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y51" t="inlineStr"/>
+      <c r="Z51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AB51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC51" t="inlineStr"/>
+      <c r="AD51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE51" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AF51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG51" t="inlineStr">
+        <is>
+          <t>Plan operativo formulado oportunamente</t>
+        </is>
+      </c>
+      <c r="AH51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI51" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK51" t="inlineStr">
+        <is>
+          <t>No se encuentra ninguna observación</t>
+        </is>
+      </c>
+      <c r="AL51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>8 GESTION DE TECNOLOGÍAS DE LA INFORMACIÓN Y COMUNICACIONES</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>7 Seguridad Digital</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>60.00%</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Ejecutar las actividades definidas para la vigencia del modelo de seguridad y privacidad de la información (MSP1) según cronograma</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Modelo de seguridad y privacidad de la información implementado para la vigencia 2025</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="K52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M52" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="O52" t="n">
+        <v>0</v>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="Q52" t="n">
+        <v>0</v>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="X52" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y52" t="inlineStr"/>
+      <c r="Z52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="AB52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC52" t="inlineStr"/>
+      <c r="AD52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE52" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="AF52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG52" t="inlineStr">
+        <is>
+          <t>Se solicitó lineamientos del MSPI a la JOTIC mediante memorandos: 20251-V-BOG-030838 y 20251-V-BOG-043356</t>
+        </is>
+      </c>
+      <c r="AH52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI52" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK52" t="inlineStr">
+        <is>
+          <t>No se encuentra ninguna observación</t>
+        </is>
+      </c>
+      <c r="AL52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>8 GESTIÓN DE TECNOLOGÍAS DE LA INFORMACIÓN Y COMUNICACIONES</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>9 Racionalización de Tramites</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>60.00%</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Apoyo técnico en la implementación de la estrategia de racionalización de trámites según plan de trabajo</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Apoyo técnico en la Estrategia de racionalización implementada y con informes de seguimiento trimestral</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="K53" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>0</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="O53" t="n">
+        <v>0</v>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="Q53" t="n">
+        <v>0</v>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>EDGAR ALEJANDRO CAMACHO MARTINEZ NESTOR ALFONSO NAVARRO TOVAR JUDY GIOVANNA BALLESTEROS BENITEZ VICTOR FERNEY HERNANDEZ AYA</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="X53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y53" t="inlineStr"/>
+      <c r="Z53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="AB53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC53" t="inlineStr"/>
+      <c r="AD53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE53" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="AF53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG53" t="inlineStr">
+        <is>
+          <t>Se realizaron pruebas en aplicativo invidentes con el permiso para la movilización de carga extraordinario por vías de acceso</t>
+        </is>
+      </c>
+      <c r="AH53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI53" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK53" t="inlineStr">
+        <is>
+          <t>No se encuentra ninguna observación</t>
+        </is>
+      </c>
+      <c r="AL53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>9 ATENCION Y RELACIONAMIENTO AL CIUDADANO</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>49 Servicio al ciudadano</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>75.00%</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Atender las peticiones, quejas, reclamos y denuncias (PQRD) de acuerdo a ley y demás disposiciones vigentes</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>PQRD atendidas de acuerdo a ley y demás disposiciones vigentes</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K54" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M54" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O54" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q54" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>EDGAR ALEJANDRO CAMACHO MARTINEZ GLADYS GUTIERREZ ZULUAGA JOSE LUIS ESCOBAR ROJAS DAVID RICARDO PEREZ MORENO JULI CATHERINE RULLE ESPARROS BENITEZ VICTOR FERNEY MERCADEZ AYA ERVIN FELIPE PADILLA LOZANO JUAN JOSE LOPEZ MENDOZA BRYAN GILDARDO OLAYA YATE</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y54" t="inlineStr"/>
+      <c r="Z54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC54" t="inlineStr"/>
+      <c r="AD54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE54" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG54" t="inlineStr">
+        <is>
+          <t>PQRD atendidas oportunamente</t>
+        </is>
+      </c>
+      <c r="AH54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI54" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK54" t="inlineStr">
+        <is>
+          <t>No se encuetra ninguna observación</t>
+        </is>
+      </c>
+      <c r="AL54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>9 ATENCION Y RELACIONAMIENTO AL CIUDADANO</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>50 Participación ciudadana en la gestión pública</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>75.00%</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Implementar la estrategia de participación ciudadana</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Estrategia de participación ciudadana aprobada, implementada y con seguimiento</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K55" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O55" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q55" t="n">
+        <v>0</v>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="X55" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y55" t="inlineStr"/>
+      <c r="Z55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC55" t="inlineStr"/>
+      <c r="AD55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE55" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG55" t="inlineStr"/>
+      <c r="AH55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI55" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK55" t="inlineStr"/>
+      <c r="AL55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>13 DIRECCIONAMIENTO ESTRATÉGICO Y PLANEACIÓN INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2 Fortalecimiento organizacional y simplificación de procesos</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Revisar y actualizar mejoras cuando sea el caso de la documentación de los procesos del Modelo de Operación</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Procesos del Modelo de Operación revisados y si se requieren mejorados</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="K56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Q56" t="n">
+        <v>0</v>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X56" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y56" t="inlineStr"/>
+      <c r="Z56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA56" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC56" t="inlineStr"/>
+      <c r="AD56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE56" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="AF56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG56" t="inlineStr"/>
+      <c r="AH56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI56" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK56" t="inlineStr"/>
+      <c r="AL56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>11 EVALUACION Y SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>28 Seguimiento y evaluación del desempeño institucional</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>75.00%</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Evaluar plan operativo</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Plan operativo evaluado</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M57" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O57" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q57" t="n">
+        <v>0</v>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X57" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y57" t="inlineStr"/>
+      <c r="Z57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC57" t="inlineStr"/>
+      <c r="AD57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE57" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG57" t="inlineStr"/>
+      <c r="AH57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI57" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK57" t="inlineStr"/>
+      <c r="AL57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>13 DIRECCIONAMIENTO ESTRATÉGICO Y PLANEACIÓN INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>105 Seguimiento y evaluación del desempeño institucional</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Gestionar las solicitudes de los permisos de cierres de via por evento deportivos o culturales, por obra y por emergencia</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Emisión del concepto de viabilidad</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K58" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M58" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O58" t="n">
+        <v>0</v>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q58" t="n">
+        <v>0</v>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>JULY CATHERINE BALLESTEROS BENITEZ</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="X58" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y58" t="inlineStr"/>
+      <c r="Z58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC58" t="inlineStr"/>
+      <c r="AD58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE58" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG58" t="inlineStr"/>
+      <c r="AH58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI58" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK58" t="inlineStr"/>
+      <c r="AL58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>13 DIRECCIONAMIENTO ESTRATÉGICO Y PLANEACIÓN INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>105 Seguimiento y evaluación del desempeño institucional</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Gestionar las solicitudes para la expedición de los permisos para la movilización de carga indivisible, extrappesada, indivisible extradimensionada o indivisible extrappesada y extradimensionada a la vez y permiso de transporte de carga divisible con vehículos combinados de carga VCC</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Emisión concepto de viabilidad</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M59" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O59" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q59" t="n">
+        <v>0</v>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>VICTOR FERNEY HERNANDEZ AYA ERVIN FELIPE PADILLA LOZANO JOSE LOPEZ MENDOZA</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X59" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y59" t="inlineStr"/>
+      <c r="Z59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC59" t="inlineStr"/>
+      <c r="AD59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE59" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG59" t="inlineStr"/>
+      <c r="AH59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI59" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK59" t="inlineStr"/>
+      <c r="AL59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>3</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>13 DIRECCIONAMIENTO ESTRATÉGICO Y PLANEACIÓN INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>105 Seguimiento y evaluación del desempeño institucional</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Revisión de conceptos de viabilidad frente al cumplimiento de los requisitos para el otorgamiento de permisos de movilización de carga indivisible Extrapesada, indivisible extradimensionada o indivisible extrappesada y extradimensionada a la vez y permiso de transporte de carga divisible con vehículos combinados de carga VCC, uso de zona de carreteras, cierres viales y eventos deportivos y emergencias, concepto técnico de ubicación de estaciones de servicio, previo concepto de viabilidad de la DT</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>revisión de conceptos</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="K60" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O60" t="n">
+        <v>0</v>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q60" t="n">
+        <v>0</v>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>JOSE LUIS ESCOBAR ROJAS</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X60" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y60" t="inlineStr"/>
+      <c r="Z60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC60" t="inlineStr"/>
+      <c r="AD60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE60" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG60" t="inlineStr"/>
+      <c r="AH60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI60" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK60" t="inlineStr"/>
+      <c r="AL60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>3</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>13 DIRECCIONAMIENTO ESTRATÉGICO Y PLANEACIÓN INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>105 Seguimiento y evaluación del desempeño institucional</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Atender requerimientos relacionados con la normatividad asociada a los trámites de permisos que se adelantan en la subdirección</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Plan anticorrupción y de atención al ciudadano</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="K61" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M61" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q61" t="n">
+        <v>0</v>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>JOSE LUIS ESCOBAR ROJAS</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X61" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y61" t="inlineStr"/>
+      <c r="Z61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC61" t="inlineStr"/>
+      <c r="AD61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE61" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG61" t="inlineStr"/>
+      <c r="AH61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI61" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK61" t="inlineStr"/>
+      <c r="AL61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>3</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>13 DIRECCIONAMIENTO ESTRATÉGICO Y PLANEACIÓN INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>105 Seguimiento y evaluación del desempeño institucional</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Gestionar las solicitudes para la autorización para la construcción de obras en las franjas de los ríos o dentro de su cauce y en las demás vías fluviales a cargo del Instituto Nacional de Vías</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Emisión concepto de viabilidad</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K62" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M62" t="n">
+        <v>0</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q62" t="n">
+        <v>0</v>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>DAVID RICARDO PEREZ MORENO BRYAN GILDARDO OLAYA YATE</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X62" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y62" t="inlineStr"/>
+      <c r="Z62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC62" t="inlineStr"/>
+      <c r="AD62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE62" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG62" t="inlineStr"/>
+      <c r="AH62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI62" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK62" t="inlineStr"/>
+      <c r="AL62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>13 DIRECCIONAMIENTO ESTRATÉGICO Y PLANEACIÓN INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>105 Seguimiento y evaluación del desempeño institucional</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Trámite para concepto técnico de ubicación de estaciones de servicio</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Emisión concepto</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M63" t="n">
+        <v>0</v>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O63" t="n">
+        <v>0</v>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q63" t="n">
+        <v>0</v>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>VICTOR FERNEY HERNANDEZ AYA ERVIN FELIPE PADILLA LOZANO</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X63" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y63" t="inlineStr"/>
+      <c r="Z63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC63" t="inlineStr"/>
+      <c r="AD63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE63" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG63" t="inlineStr"/>
+      <c r="AH63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI63" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK63" t="inlineStr"/>
+      <c r="AL63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>3</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>13 DIRECCIONAMIENTO ESTRATÉGICO Y PLANEACIÓN INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>105 Seguimiento y evaluación del desempeño institucional</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Gestionar la revisión de documentos de los permisos de carga extradimensionada -Revisión de documentos diario realizado en el aplicativo INVITRAMITE</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Revisión documental</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K64" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M64" t="n">
+        <v>0</v>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O64" t="n">
+        <v>0</v>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q64" t="n">
+        <v>0</v>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>EDGAR ALEJANDRO CAMACHO MARTINEZ</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X64" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y64" t="inlineStr"/>
+      <c r="Z64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC64" t="inlineStr"/>
+      <c r="AD64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE64" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG64" t="inlineStr"/>
+      <c r="AH64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI64" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK64" t="inlineStr"/>
+      <c r="AL64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>3</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>13 DIRECCIONAMIENTO ESTRATÉGICO Y PLANEACIÓN INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>105 Seguimiento y evaluación del desempeño institucional</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Gestionar solicitudes para los permisos de uso de zona de vía</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>emisión concepto de viabilidad</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K65" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M65" t="n">
+        <v>0</v>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O65" t="n">
+        <v>0</v>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q65" t="n">
+        <v>0</v>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>DAVID RICARDO PEREZ MORENO ERVIN FELIPE PADILLA LOZANO BRYAN GILDARDO OLAYA YATE</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X65" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y65" t="inlineStr"/>
+      <c r="Z65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC65" t="inlineStr"/>
+      <c r="AD65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE65" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG65" t="inlineStr"/>
+      <c r="AH65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI65" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK65" t="inlineStr"/>
+      <c r="AL65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>3</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>13 DIRECCIONAMIENTO ESTRATÉGICO Y PLANEACIÓN INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>105 Seguimiento y evaluación del desempeño institucional</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Apoyar actividades para implementar las acciones del Programa de Transparencia Ética Pública</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Acciones del Programa de Transparencia y ética pública implementadas</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M66" t="n">
+        <v>0</v>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O66" t="n">
+        <v>0</v>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q66" t="n">
+        <v>0</v>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X66" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y66" t="inlineStr"/>
+      <c r="Z66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC66" t="inlineStr"/>
+      <c r="AD66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE66" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG66" t="inlineStr"/>
+      <c r="AH66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI66" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK66" t="inlineStr"/>
+      <c r="AL66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>5 GESTION DOCUMENTAL</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>75 Gestión documental</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>75.00%</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Crear y mantener actualizados los expedientes electrónicos de la etapa precontractual de los contratos suscritos 2024, entregando los documentos para su cargue en el aplicativo AZ Digital, conforme al cumplimiento de cada instancia o trámite contractual y según plan de trabajo</t>
+        </is>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>expedientes electrónicos de la etapa precontractual de los contratos 2024 creados y actualizados y cargados en el aplicativo AZ</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K67" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O67" t="n">
+        <v>0</v>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q67" t="n">
+        <v>0</v>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="X67" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y67" t="inlineStr"/>
+      <c r="Z67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC67" t="inlineStr"/>
+      <c r="AD67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE67" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG67" t="inlineStr"/>
+      <c r="AH67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI67" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK67" t="inlineStr"/>
+      <c r="AL67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>5 GESTION DOCUMENTAL</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>75 Gestión documental</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>75.00%</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Crear y mantener actualizados los expedientes electrónicos de los contratos suscritos en la vigencia 2025, entregando los documentos para su cargue en el aplicativo AZ Digital, conforme al cumplimiento de cada instancia o trámite contractual y según plan de trabajo</t>
+        </is>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>expedientes electrónicos los contratos 2025 creados y actualizados y cargados en el aplicativo AZ</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K68" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M68" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O68" t="n">
+        <v>0</v>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q68" t="n">
+        <v>0</v>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="X68" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y68" t="inlineStr"/>
+      <c r="Z68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC68" t="inlineStr"/>
+      <c r="AD68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE68" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG68" t="inlineStr"/>
+      <c r="AH68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI68" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK68" t="inlineStr"/>
+      <c r="AL68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>4</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>11 EVALUACION Y SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>1 Control interno</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Formular e implementar el Mapa de aseguramiento y realizar reporte</t>
+        </is>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Mapa de aseguramiento formulado e implementado y reporte realizado</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K69" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M69" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O69" t="n">
+        <v>0</v>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q69" t="n">
+        <v>0</v>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR JOSE LUIS ESCOBAR ROJAS</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y69" t="inlineStr"/>
+      <c r="Z69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC69" t="inlineStr"/>
+      <c r="AD69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE69" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG69" t="inlineStr">
+        <is>
+          <t>Mapa de aseguramiento remitido a la oficina de control internoObserva 4°Trimestre: No se encuentra ninguna observación</t>
+        </is>
+      </c>
+      <c r="AH69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI69" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK69" t="inlineStr"/>
+      <c r="AL69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>datos/Siplan- Grupo permisos.pdf</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>4</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>11 EVALUACION Y SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>1 Control interno</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Formular, implementar y reportar cumplimiento de los planes de mejoramiento de auditorias internas y externas</t>
+        </is>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Planes de mejoramiento de auditorias internas y externas formulados, implementados y con reporte de cumplimiento</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="K70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="M70" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="O70" t="n">
+        <v>0</v>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="Q70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>NESTOR ALFONSO NAVARRO TOVAR</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="X70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y70" t="inlineStr"/>
+      <c r="Z70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="AB70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC70" t="inlineStr"/>
+      <c r="AD70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE70" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="AF70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG70" t="inlineStr"/>
+      <c r="AH70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI70" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="AJ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK70" t="inlineStr"/>
+      <c r="AL70" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>